<commit_message>
added all Transaction overivew with Line chart
</commit_message>
<xml_diff>
--- a/backend/all_transactions.xlsx
+++ b/backend/all_transactions.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D14"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -419,13 +419,13 @@
     </row>
     <row r="2">
       <c r="A2" s="1">
-        <v>45853.22928240741</v>
+        <v>45861.22928240741</v>
       </c>
       <c r="B2" t="str">
         <v>Expense</v>
       </c>
       <c r="C2" t="str">
-        <v>food</v>
+        <v>Banana</v>
       </c>
       <c r="D2">
         <v>100</v>
@@ -433,27 +433,27 @@
     </row>
     <row r="3">
       <c r="A3" s="1">
-        <v>45847.22928240741</v>
+        <v>45853.22928240741</v>
       </c>
       <c r="B3" t="str">
         <v>Income</v>
       </c>
       <c r="C3" t="str">
-        <v>Cashback</v>
+        <v>BSCC</v>
       </c>
       <c r="D3">
-        <v>500</v>
+        <v>5000</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1">
-        <v>45847.22928240741</v>
+        <v>45853.22928240741</v>
       </c>
       <c r="B4" t="str">
         <v>Expense</v>
       </c>
       <c r="C4" t="str">
-        <v>Juice</v>
+        <v>food</v>
       </c>
       <c r="D4">
         <v>100</v>
@@ -464,97 +464,97 @@
         <v>45847.22928240741</v>
       </c>
       <c r="B5" t="str">
-        <v>Expense</v>
+        <v>Income</v>
       </c>
       <c r="C5" t="str">
-        <v>Mutton</v>
+        <v>Cashback</v>
       </c>
       <c r="D5">
-        <v>250</v>
+        <v>500</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1">
-        <v>45844.22928240741</v>
+        <v>45847.22928240741</v>
       </c>
       <c r="B6" t="str">
-        <v>Income</v>
+        <v>Expense</v>
       </c>
       <c r="C6" t="str">
-        <v>Bug Fixed</v>
+        <v>Juice</v>
       </c>
       <c r="D6">
-        <v>10000</v>
+        <v>100</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1">
-        <v>45844.22928240741</v>
+        <v>45847.22928240741</v>
       </c>
       <c r="B7" t="str">
         <v>Expense</v>
       </c>
       <c r="C7" t="str">
-        <v>footwear</v>
+        <v>Mutton</v>
       </c>
       <c r="D7">
-        <v>200</v>
+        <v>250</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1">
-        <v>45843.22928240741</v>
+        <v>45844.22928240741</v>
       </c>
       <c r="B8" t="str">
         <v>Income</v>
       </c>
       <c r="C8" t="str">
-        <v>Bussiness</v>
+        <v>Bug Fixed</v>
       </c>
       <c r="D8">
-        <v>1000</v>
+        <v>10000</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1">
-        <v>45843.22928240741</v>
+        <v>45844.22928240741</v>
       </c>
       <c r="B9" t="str">
-        <v>Income</v>
+        <v>Expense</v>
       </c>
       <c r="C9" t="str">
-        <v>Apps</v>
+        <v>footwear</v>
       </c>
       <c r="D9">
-        <v>500</v>
+        <v>200</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1">
-        <v>45842.22928240741</v>
+        <v>45843.22928240741</v>
       </c>
       <c r="B10" t="str">
-        <v>Expense</v>
+        <v>Income</v>
       </c>
       <c r="C10" t="str">
-        <v>food</v>
+        <v>Bussiness</v>
       </c>
       <c r="D10">
-        <v>120</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1">
-        <v>45840.79550543981</v>
+        <v>45843.22928240741</v>
       </c>
       <c r="B11" t="str">
         <v>Income</v>
       </c>
       <c r="C11" t="str">
-        <v>Salary</v>
+        <v>Apps</v>
       </c>
       <c r="D11">
-        <v>6000</v>
+        <v>500</v>
       </c>
     </row>
     <row r="12">
@@ -562,39 +562,53 @@
         <v>45840.79550543981</v>
       </c>
       <c r="B12" t="str">
-        <v>Expense</v>
+        <v>Income</v>
       </c>
       <c r="C12" t="str">
-        <v>rent</v>
+        <v>Salary</v>
       </c>
       <c r="D12">
-        <v>500</v>
+        <v>6000</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1">
-        <v>45827.22928240741</v>
+        <v>45840.79550543981</v>
       </c>
       <c r="B13" t="str">
         <v>Expense</v>
       </c>
       <c r="C13" t="str">
+        <v>rent</v>
+      </c>
+      <c r="D13">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1">
+        <v>45827.22928240741</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Expense</v>
+      </c>
+      <c r="C14" t="str">
         <v>house</v>
       </c>
-      <c r="D13">
+      <c r="D14">
         <v>1000</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D13"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D14"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C7"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -609,35 +623,35 @@
     </row>
     <row r="2">
       <c r="A2" s="1">
-        <v>45847.22928240741</v>
+        <v>45853.22928240741</v>
       </c>
       <c r="B2" t="str">
-        <v>Cashback</v>
+        <v>BSCC</v>
       </c>
       <c r="C2">
-        <v>500</v>
+        <v>5000</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1">
-        <v>45844.22928240741</v>
+        <v>45847.22928240741</v>
       </c>
       <c r="B3" t="str">
-        <v>Bug Fixed</v>
+        <v>Cashback</v>
       </c>
       <c r="C3">
-        <v>10000</v>
+        <v>500</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1">
-        <v>45843.22928240741</v>
+        <v>45844.22928240741</v>
       </c>
       <c r="B4" t="str">
-        <v>Bussiness</v>
+        <v>Bug Fixed</v>
       </c>
       <c r="C4">
-        <v>1000</v>
+        <v>10000</v>
       </c>
     </row>
     <row r="5">
@@ -645,26 +659,37 @@
         <v>45843.22928240741</v>
       </c>
       <c r="B5" t="str">
-        <v>Apps</v>
+        <v>Bussiness</v>
       </c>
       <c r="C5">
-        <v>500</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1">
+        <v>45843.22928240741</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Apps</v>
+      </c>
+      <c r="C6">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1">
         <v>45840.79550543981</v>
       </c>
-      <c r="B6" t="str">
+      <c r="B7" t="str">
         <v>Salary</v>
       </c>
-      <c r="C6">
+      <c r="C7">
         <v>6000</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C7"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -686,10 +711,10 @@
     </row>
     <row r="2">
       <c r="A2" s="1">
-        <v>45853.22928240741</v>
+        <v>45861.22928240741</v>
       </c>
       <c r="B2" t="str">
-        <v>food</v>
+        <v>Banana</v>
       </c>
       <c r="C2">
         <v>100</v>
@@ -697,10 +722,10 @@
     </row>
     <row r="3">
       <c r="A3" s="1">
-        <v>45847.22928240741</v>
+        <v>45853.22928240741</v>
       </c>
       <c r="B3" t="str">
-        <v>Juice</v>
+        <v>food</v>
       </c>
       <c r="C3">
         <v>100</v>
@@ -711,32 +736,32 @@
         <v>45847.22928240741</v>
       </c>
       <c r="B4" t="str">
-        <v>Mutton</v>
+        <v>Juice</v>
       </c>
       <c r="C4">
-        <v>250</v>
+        <v>100</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1">
-        <v>45844.22928240741</v>
+        <v>45847.22928240741</v>
       </c>
       <c r="B5" t="str">
-        <v>footwear</v>
+        <v>Mutton</v>
       </c>
       <c r="C5">
-        <v>200</v>
+        <v>250</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1">
-        <v>45842.22928240741</v>
+        <v>45844.22928240741</v>
       </c>
       <c r="B6" t="str">
-        <v>food</v>
+        <v>footwear</v>
       </c>
       <c r="C6">
-        <v>120</v>
+        <v>200</v>
       </c>
     </row>
     <row r="7">
@@ -785,7 +810,7 @@
         <v>Total Income</v>
       </c>
       <c r="B2">
-        <v>18000</v>
+        <v>23000</v>
       </c>
     </row>
     <row r="3">
@@ -793,7 +818,7 @@
         <v>Total Expenses</v>
       </c>
       <c r="B3">
-        <v>2270</v>
+        <v>2250</v>
       </c>
     </row>
     <row r="4">
@@ -801,7 +826,7 @@
         <v>Net Balance</v>
       </c>
       <c r="B4">
-        <v>15730</v>
+        <v>20750</v>
       </c>
     </row>
     <row r="5">
@@ -809,7 +834,7 @@
         <v>Total Transactions</v>
       </c>
       <c r="B5">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="6">
@@ -817,7 +842,7 @@
         <v>Income Transactions</v>
       </c>
       <c r="B6">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7">

</xml_diff>